<commit_message>
Fix: Corrigir importação de dados de comissionistas 2026
- Março 2026 estava com valores errados (€25.174 em vez de €3.332)
- Janeiro e Fevereiro 2026 também tinham valores multiplicados incorretamente
- Problema: script antigo usava pandas e multiplicava dias × preço
- Solução: reimportar com openpyxl usando preço direto da coluna D (Loyalty Card)
- Todos os dados de Jan, Fev e Mar 2026 agora corretos
- Adicionar scripts de verificação e correção
</commit_message>
<xml_diff>
--- a/CM-03-2026.xlsx
+++ b/CM-03-2026.xlsx
@@ -5,22 +5,35 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filipepacheco/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filipepacheco/CascadeProjects/carscraping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88E13B2D-84D2-FC47-BEC9-C17743138759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D31818-0F60-0842-9932-9AB8731C1D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15960" xr2:uid="{82174858-6960-624C-A441-23BE34989D8B}"/>
+    <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15900" xr2:uid="{82174858-6960-624C-A441-23BE34989D8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Loyalty Card" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="90">
   <si>
     <t>Voucher</t>
   </si>
@@ -55,42 +68,15 @@
     <t>3</t>
   </si>
   <si>
-    <t>170</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
     <t>2026-03-03 10:00:00</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>85</t>
-  </si>
-  <si>
-    <t>65</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
     <t>2026-03-15 16:00:00</t>
   </si>
   <si>
@@ -100,9 +86,6 @@
     <t>2026-03-18 15:00:00</t>
   </si>
   <si>
-    <t>75</t>
-  </si>
-  <si>
     <t>2026-03-27 09:30:00</t>
   </si>
   <si>
@@ -133,9 +116,6 @@
     <t>2026-03-05 10:30:00</t>
   </si>
   <si>
-    <t>160</t>
-  </si>
-  <si>
     <t>2026-03-13 10:00:00</t>
   </si>
   <si>
@@ -148,33 +128,21 @@
     <t>2026-03-06 11:00:00</t>
   </si>
   <si>
-    <t>23,76</t>
-  </si>
-  <si>
     <t>D013231033-4PUJ</t>
   </si>
   <si>
-    <t>84,72</t>
-  </si>
-  <si>
     <t>D013271768-PMEV</t>
   </si>
   <si>
     <t>2026-03-21 11:00:00</t>
   </si>
   <si>
-    <t>101,04</t>
-  </si>
-  <si>
     <t>D013457069-X5SN</t>
   </si>
   <si>
     <t>2026-03-31 11:00:00</t>
   </si>
   <si>
-    <t>52,82</t>
-  </si>
-  <si>
     <t>EPIC SANA</t>
   </si>
   <si>
@@ -223,9 +191,6 @@
     <t>2026-03-27 10:45:00</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
     <t>2026-03-30 11:00:00</t>
   </si>
   <si>
@@ -262,9 +227,6 @@
     <t>2026-03-04 09:30:00</t>
   </si>
   <si>
-    <t>90</t>
-  </si>
-  <si>
     <t>OURA VIEW BEACH CLUB</t>
   </si>
   <si>
@@ -274,9 +236,6 @@
     <t>PALADIM</t>
   </si>
   <si>
-    <t>120</t>
-  </si>
-  <si>
     <t>PATEO VILLAGE</t>
   </si>
   <si>
@@ -292,9 +251,6 @@
     <t>2026-03-07 10:15:00</t>
   </si>
   <si>
-    <t>35</t>
-  </si>
-  <si>
     <t>PTO</t>
   </si>
   <si>
@@ -338,9 +294,6 @@
   </si>
   <si>
     <t>SOL E MAR</t>
-  </si>
-  <si>
-    <t>130</t>
   </si>
   <si>
     <t>ZEBRA SAFARIS II</t>
@@ -848,7 +801,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -862,6 +815,17 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Cor1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1237,16 +1201,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4882FE-6D1D-AD42-8DFC-F61752C98768}">
-  <dimension ref="A1:D276"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G86"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1256,299 +1220,300 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D3" s="7">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D4" s="8"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D6" s="7">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D7" s="7">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D8" s="7">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D9" s="8"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D11" s="7">
+        <v>23.76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D12" s="7">
+        <v>84.72</v>
+      </c>
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D13" s="7">
+        <v>101.04</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D14" s="7">
+        <v>52.82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D15" s="8"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D17" s="7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D18" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="3" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D19" s="7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D20" s="8"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D22" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D23" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D24" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D25" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D26" s="7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D27" s="8"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
     </row>
-    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="3" t="s">
         <v>6</v>
@@ -1556,766 +1521,585 @@
       <c r="C29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D29" s="7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="3" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D30" s="7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="3" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D31" s="7">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="3" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D32" s="7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="3" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D33" s="7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D34" s="8"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
     </row>
-    <row r="36" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="3" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D36" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D37" s="8"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
     </row>
-    <row r="39" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="3" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D39" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D40" s="8"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
     </row>
-    <row r="42" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="3" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D42" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-    </row>
-    <row r="44" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D43" s="8"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
     </row>
-    <row r="45" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="3" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D45" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D45" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-    </row>
-    <row r="47" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D46" s="8"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
     </row>
-    <row r="48" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D48" s="7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D49" s="8"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
     </row>
-    <row r="51" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="3" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D51" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D51" s="7">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D52" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-    </row>
-    <row r="54" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
     </row>
-    <row r="55" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="3" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D55" s="7">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-    </row>
-    <row r="57" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D56" s="8"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
     </row>
-    <row r="58" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D58" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D58" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-    </row>
-    <row r="60" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D59" s="8"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
     </row>
-    <row r="61" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="3" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D61" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D61" s="7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="3" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D62" s="7">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="3" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D63" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D63" s="7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="3" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+      <c r="D64" s="7">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D65" s="8"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
     </row>
-    <row r="67" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D67" s="7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D68" s="7">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D69" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D70" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D70" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="3" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B72" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D72" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D72" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-    </row>
-    <row r="74" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D73" s="8"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
     </row>
-    <row r="75" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="3" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+      <c r="D75" s="7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="3" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D76" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D76" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="3" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D77" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D77" s="7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="3" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D78" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D78" s="7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-    </row>
-    <row r="80" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D79" s="8"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
     </row>
-    <row r="81" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="3" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D81" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D81" s="7">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-    </row>
-    <row r="83" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D82" s="8"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
     </row>
-    <row r="84" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D84" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D84" s="7">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D85" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="D85" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="88" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="89" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="90" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="91" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="92" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="93" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="94" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="96" spans="1:4" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="113" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="114" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="115" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="116" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="117" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="118" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="119" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="120" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="121" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="122" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="123" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="124" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="125" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="126" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="127" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="128" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="129" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="130" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="131" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="132" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="133" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="134" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="135" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="136" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="137" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="138" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="139" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="140" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="141" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="142" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="143" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="144" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="145" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="146" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="147" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="148" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="149" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="150" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="151" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="152" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="153" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="154" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="155" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="156" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="157" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="158" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="159" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="160" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="161" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="162" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="163" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="164" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="165" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="166" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="167" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="168" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="169" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="170" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="171" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="172" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="173" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="174" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="175" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="176" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="177" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="178" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="179" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="180" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="181" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="182" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="183" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="184" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="185" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="186" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="187" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="188" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="189" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="190" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="191" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="192" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="193" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="194" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="195" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="196" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="197" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="198" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="199" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="200" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="201" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="202" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="203" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="204" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="205" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="206" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="207" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="208" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="209" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="210" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="211" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="212" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="213" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="214" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="215" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="216" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="217" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="218" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="219" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="220" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="221" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="222" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="223" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="224" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="225" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="226" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="227" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="228" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="229" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="230" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="231" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="232" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="233" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="234" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="235" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="236" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="237" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="238" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="239" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="240" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="241" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="242" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="243" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="244" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="245" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="246" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="247" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="248" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="249" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="250" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="251" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="252" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="253" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="254" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="255" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="256" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="257" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="258" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="259" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="260" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="261" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="262" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="263" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="264" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="265" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="266" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="267" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="268" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="269" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="270" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="271" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="272" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="273" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="274" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="275" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="276" ht="12" x14ac:dyDescent="0.2"/>
+      <c r="D86" s="8"/>
+    </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A38:D38"/>
     <mergeCell ref="A66:D66"/>
     <mergeCell ref="A74:D74"/>
     <mergeCell ref="A80:D80"/>
@@ -2326,15 +2110,6 @@
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A57:D57"/>
     <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Excel upload button for commission imports - uses current year with month/day from file
</commit_message>
<xml_diff>
--- a/CM-03-2026.xlsx
+++ b/CM-03-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filipepacheco/CascadeProjects/carscraping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D31818-0F60-0842-9932-9AB8731C1D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92F63810-A310-2C48-A5FB-74A632352836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15900" xr2:uid="{82174858-6960-624C-A441-23BE34989D8B}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>Voucher</t>
   </si>
@@ -59,9 +59,6 @@
     <t>6</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -117,30 +114,6 @@
   </si>
   <si>
     <t>2026-03-13 10:00:00</t>
-  </si>
-  <si>
-    <t>DISCOVERCARS-PREPAID</t>
-  </si>
-  <si>
-    <t>D013233923-NN5R</t>
-  </si>
-  <si>
-    <t>2026-03-06 11:00:00</t>
-  </si>
-  <si>
-    <t>D013231033-4PUJ</t>
-  </si>
-  <si>
-    <t>D013271768-PMEV</t>
-  </si>
-  <si>
-    <t>2026-03-21 11:00:00</t>
-  </si>
-  <si>
-    <t>D013457069-X5SN</t>
-  </si>
-  <si>
-    <t>2026-03-31 11:00:00</t>
   </si>
   <si>
     <t>EPIC SANA</t>
@@ -801,7 +774,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -812,10 +785,6 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -826,6 +795,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Cor1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1201,16 +1173,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4882FE-6D1D-AD42-8DFC-F61752C98768}">
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1220,382 +1192,363 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="7">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5">
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="8"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="7">
+        <v>12</v>
+      </c>
+      <c r="D7" s="5">
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="7">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5">
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="8"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2"/>
+      <c r="B11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="C11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2"/>
+      <c r="B12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="7">
-        <v>23.76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="B16" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="7">
-        <v>84.72</v>
-      </c>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="D17" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2"/>
+      <c r="B23" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="7">
-        <v>101.04</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="7">
-        <v>52.82</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="8"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="7">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="7">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="D23" s="5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="2"/>
+      <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="2"/>
+      <c r="B25" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="3" t="s">
+      <c r="D25" s="5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="2"/>
+      <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="7">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="C26" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="7">
-        <v>70</v>
+        <v>9</v>
+      </c>
+      <c r="D26" s="5">
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="8"/>
+      <c r="B27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="5">
+        <v>75</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="7">
-        <v>80</v>
-      </c>
+      <c r="A29" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D30" s="7">
-        <v>80</v>
+      <c r="D30" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="7">
-        <v>60</v>
-      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="6"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="2"/>
-      <c r="B32" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="7">
-        <v>75</v>
-      </c>
+      <c r="A32" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="7">
-        <v>75</v>
+        <v>9</v>
+      </c>
+      <c r="D33" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="8"/>
+      <c r="D34" s="6"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
+      <c r="A35" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="7">
+        <v>9</v>
+      </c>
+      <c r="D36" s="5">
         <v>50</v>
       </c>
     </row>
@@ -1603,513 +1556,460 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="8"/>
+      <c r="D37" s="6"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
+      <c r="A38" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="7">
-        <v>50</v>
+        <v>9</v>
+      </c>
+      <c r="D39" s="5">
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="8"/>
+      <c r="D40" s="6"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
+      <c r="A41" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D42" s="7">
-        <v>50</v>
+        <v>8</v>
+      </c>
+      <c r="D42" s="5">
+        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
-      <c r="D43" s="8"/>
+      <c r="D43" s="6"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
+      <c r="A44" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="7">
-        <v>100</v>
+        <v>5</v>
+      </c>
+      <c r="D45" s="5">
+        <v>65</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="8"/>
+      <c r="B46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="5">
+        <v>45</v>
+      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="6"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="2"/>
-      <c r="B48" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48" s="7">
-        <v>90</v>
-      </c>
+      <c r="A48" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="8"/>
+      <c r="B49" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D49" s="5">
+        <v>120</v>
+      </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="6"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="2"/>
-      <c r="B51" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D51" s="7">
-        <v>65</v>
-      </c>
+      <c r="A51" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="2"/>
+      <c r="A52" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="B52" s="3" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D52" s="7">
-        <v>45</v>
+        <v>9</v>
+      </c>
+      <c r="D52" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="8"/>
+      <c r="D53" s="6"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
+      <c r="A54" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D55" s="7">
-        <v>120</v>
+        <v>9</v>
+      </c>
+      <c r="D55" s="5">
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="8"/>
+      <c r="B56" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" s="5">
+        <v>60</v>
+      </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
+      <c r="A57" s="2"/>
+      <c r="B57" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D57" s="5">
+        <v>70</v>
+      </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="3" t="s">
-        <v>68</v>
-      </c>
+      <c r="A58" s="2"/>
       <c r="B58" s="3" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D58" s="7">
-        <v>50</v>
+      <c r="D58" s="5">
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
-      <c r="D59" s="8"/>
+      <c r="D59" s="6"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" s="5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D63" s="5">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="2"/>
-      <c r="B61" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D61" s="7">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="2"/>
-      <c r="B62" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D62" s="7">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="2"/>
-      <c r="B63" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D63" s="7">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="2"/>
       <c r="B64" s="3" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" s="7">
-        <v>35</v>
+        <v>9</v>
+      </c>
+      <c r="D64" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="8"/>
+      <c r="B65" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" s="5">
+        <v>45</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="4" t="s">
+      <c r="A66" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B66" s="4"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
+      <c r="B66" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="5">
+        <v>50</v>
+      </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="6"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B68" s="8"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="8"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="2"/>
+      <c r="B69" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C69" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D69" s="5">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="2"/>
+      <c r="B70" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C70" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="7">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D68" s="7">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D69" s="7">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D70" s="7">
+      <c r="D70" s="5">
         <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D71" s="7">
-        <v>45</v>
+        <v>5</v>
+      </c>
+      <c r="D71" s="5">
+        <v>90</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
-        <v>81</v>
-      </c>
+      <c r="A72" s="2"/>
       <c r="B72" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D72" s="7">
-        <v>50</v>
+        <v>9</v>
+      </c>
+      <c r="D72" s="5">
+        <v>75</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
-      <c r="D73" s="8"/>
+      <c r="D73" s="6"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B74" s="4"/>
-      <c r="C74" s="4"/>
-      <c r="D74" s="4"/>
+      <c r="A74" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B74" s="8"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="8"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="3" t="s">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D75" s="7">
-        <v>40</v>
+        <v>9</v>
+      </c>
+      <c r="D75" s="5">
+        <v>130</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
-      <c r="B76" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D76" s="7">
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="6"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B77" s="8"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="8"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D78" s="5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D79" s="5">
         <v>50</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="2"/>
-      <c r="B77" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D77" s="7">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="2"/>
-      <c r="B78" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D78" s="7">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="8"/>
-    </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B80" s="4"/>
-      <c r="C80" s="4"/>
-      <c r="D80" s="4"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="2"/>
-      <c r="B81" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D81" s="7">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="8"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B83" s="4"/>
-      <c r="C83" s="4"/>
-      <c r="D83" s="4"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D84" s="7">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D85" s="7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="8"/>
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="18">
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A38:D38"/>
     <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>